<commit_message>
Replace 12 clubs with League Champion cards
Removes Espanyol, Deportivo, Real Sociedad, Parma, Sampdoria, Hamburg,
Werder Bremen, Stuttgart, Bordeaux, Saint-Etienne, Lens and Rennes as
cards (38 clubs left) and adds a League Champion card of the same league
for each, so every league colour keeps 13 subject cards and the deck
stays at 151. Spells at the removed clubs still count for league and
coach cards.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01991RcZHLM1eRojQbRydxnP
</commit_message>
<xml_diff>
--- a/one-two/data/player-data-template.xlsx
+++ b/one-two/data/player-data-template.xlsx
@@ -599,7 +599,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Club code: pick from the list (the 50 card clubs). For any other club choose OTHER and type its name and league.</t>
+          <t xml:space="preserve">  Club code: pick from the list (the 38 card clubs). For any other club choose OTHER and type its name and league.</t>
         </is>
       </c>
     </row>
@@ -37858,7 +37858,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C3003" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$A$1:$A$51</formula1>
+      <formula1>=Lists!$A$1:$A$39</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E3003" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$B$1:$B$6</formula1>
@@ -37878,7 +37878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -38340,17 +38340,17 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>ESY</t>
+          <t>SEV</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Barcelona Blue-White</t>
+          <t>Seville White</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -38372,17 +38372,17 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>SEV</t>
+          <t>BET</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Seville White</t>
+          <t>Seville Green</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Real Betis</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -38404,17 +38404,17 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>BET</t>
+          <t>VAL</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Seville Green</t>
+          <t>Valencia White</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Real Betis</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -38436,17 +38436,17 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>VAL</t>
+          <t>VIL</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Valencia White</t>
+          <t>Castellón Yellow</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -38468,113 +38468,113 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>VIL</t>
+          <t>JUV</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Castellón Yellow</t>
+          <t>Turin Black-White</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>ESP</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>yellow</t>
+          <t>blue</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>RSO</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>San Sebastián Blue</t>
+          <t>Milan Red-Black</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>ESP</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>yellow</t>
+          <t>blue</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>DEP</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Coruña Blue</t>
+          <t>Milan Blue-Black</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Deportivo La Coruña</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>ESP</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>yellow</t>
+          <t>blue</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>JUV</t>
+          <t>ROM</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Turin Black-White</t>
+          <t>Rome Yellow-Red</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -38596,17 +38596,17 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>LAZ</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Milan Red-Black</t>
+          <t>Rome Sky</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -38628,17 +38628,17 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>NAP</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Milan Blue-Black</t>
+          <t>Naples Blue</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -38660,17 +38660,17 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>ROM</t>
+          <t>FIO</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Rome Yellow-Red</t>
+          <t>Florence Violet</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -38692,17 +38692,17 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>LAZ</t>
+          <t>ATA</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Rome Sky</t>
+          <t>Bergamo Blue</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -38724,177 +38724,177 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>NAP</t>
+          <t>BAY</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Naples Blue</t>
+          <t>Munich Red</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Bayern Munich</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>green</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>FIO</t>
+          <t>BVB</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Florence Violet</t>
+          <t>Dortmund Yellow</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Borussia Dortmund</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>green</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>ATA</t>
+          <t>LEV</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Bergamo Blue</t>
+          <t>Leverkusen Red-Black</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>green</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>S04</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Parma Yellow-Blue</t>
+          <t>Gelsenkirchen Royal</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Schalke 04</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>green</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>SAM</t>
+          <t>RBL</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Genova Hoops</t>
+          <t>Leipzig White-Red</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Sampdoria</t>
+          <t>RB Leipzig</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>green</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>BAY</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Munich Red</t>
+          <t>Wolfsburg Green</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>VfL Wolfsburg</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -38916,17 +38916,17 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>BVB</t>
+          <t>SGE</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Dortmund Yellow</t>
+          <t>Frankfurt Black-Red</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -38948,574 +38948,190 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>LEV</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Leverkusen Red-Black</t>
+          <t>Paris Blue-Red</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Paris Saint-Germain</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>GER</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>purple</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>OMR</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Gelsenkirchen Royal</t>
+          <t>Marseille Sky</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Schalke 04</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>GER</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>purple</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>RBL</t>
+          <t>LYO</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Leipzig White-Red</t>
+          <t>Lyon White</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>GER</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>purple</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>WOB</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Wolfsburg Green</t>
+          <t>Monaco Red-White</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>VfL Wolfsburg</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>GER</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>purple</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>VFB</t>
+          <t>LIL</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Stuttgart White</t>
+          <t>Lille Red</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>VfB Stuttgart</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>GER</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>purple</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>HSV</t>
+          <t>NIC</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Hamburg Blue</t>
+          <t>Nice Red-Black</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>GER</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>SVW</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>Bremen Green</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>Werder Bremen</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>GER</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>SGE</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Frankfurt Black-Red</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Eintracht Frankfurt</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>GER</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>PSG</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Paris Blue-Red</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Paris Saint-Germain</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>OMR</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>Marseille Sky</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Marseille</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>LYO</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Lyon White</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Lyon</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>MON</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Monaco Red-White</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Monaco</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>LIL</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Lille Red</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>Lille</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>BDX</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Bordeaux Navy</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>Bordeaux</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>NIC</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>Nice Red-Black</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>Nice</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>REN</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Rennes Red</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>Rennes</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>LEN</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Lens Gold</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>Lens</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>purple</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>STE</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Saint-Étienne Green</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Saint-Étienne</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
         <is>
           <t>purple</t>
         </is>
@@ -41309,7 +40925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41436,269 +41052,205 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ESY</t>
+          <t>SEV</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SEV</t>
+          <t>BET</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BET</t>
+          <t>VAL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VAL</t>
+          <t>VIL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VIL</t>
+          <t>JUV</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RSO</t>
+          <t>MIL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DEP</t>
+          <t>INT</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>JUV</t>
+          <t>ROM</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>LAZ</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>NAP</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ROM</t>
+          <t>FIO</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LAZ</t>
+          <t>ATA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NAP</t>
+          <t>BAY</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FIO</t>
+          <t>BVB</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ATA</t>
+          <t>LEV</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>S04</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAM</t>
+          <t>RBL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BAY</t>
+          <t>WOB</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BVB</t>
+          <t>SGE</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LEV</t>
+          <t>PSG</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>OMR</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RBL</t>
+          <t>LYO</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>WOB</t>
+          <t>MON</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VFB</t>
+          <t>LIL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HSV</t>
+          <t>NIC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SVW</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>SGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>PSG</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>OMR</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>LYO</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>MON</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>LIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>BDX</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>NIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>REN</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>LEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>STE</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
           <t>OTHER</t>
         </is>
       </c>
     </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>